<commit_message>
Updated some wrong graphs
</commit_message>
<xml_diff>
--- a/7_Data_Extraction/Data_Extraction_Antonio.xlsx
+++ b/7_Data_Extraction/Data_Extraction_Antonio.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11214"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://communitystudentiunina.sharepoint.com/sites/PRINMEDITATE/Shared Documents/SLR/RegressionTestingOptimizationSLR/7_Data_Extraction/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/antoniotrovato/Documents/GitHub/RegressionTestingOptimizationSLR/7_Data_Extraction/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="432" documentId="13_ncr:1_{41748892-67E4-6840-ACCF-49487A14C08A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A413E6CF-9099-FE42-A748-6057589FC52A}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AB333AA-940A-374A-836B-16F6F03ADD35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="500" windowWidth="51200" windowHeight="28300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="15540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2477,6 +2477,9 @@
       <c r="AC8" s="1" t="s">
         <v>133</v>
       </c>
+      <c r="AH8" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="9" spans="1:34" ht="192" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
@@ -4158,6 +4161,9 @@
       </c>
       <c r="Y33" s="1" t="s">
         <v>58</v>
+      </c>
+      <c r="AH33" s="1">
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:34" ht="96" x14ac:dyDescent="0.2">
@@ -4235,15 +4241,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100B6889C2593FACB4192549183B8B19287" ma:contentTypeVersion="11" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="8f919e2780f892880bff7efb43d3db1d">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="ab92c565-5003-4ac3-93a3-a3ce8796a3c0" xmlns:ns3="aa1b21cb-23df-461b-8b8e-4aaeac2f3f50" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1ca4d89da73e1329ebe7ff2e4ed471c6" ns2:_="" ns3:_="">
     <xsd:import namespace="ab92c565-5003-4ac3-93a3-a3ce8796a3c0"/>
@@ -4438,7 +4435,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="ab92c565-5003-4ac3-93a3-a3ce8796a3c0">
@@ -4449,19 +4446,35 @@
 </p:properties>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{46AEFCCE-2E3A-4CC4-B95D-A9558D3302B7}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EB7FAFA6-FDCF-4091-8393-B79695D0D663}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="ab92c565-5003-4ac3-93a3-a3ce8796a3c0"/>
+    <ds:schemaRef ds:uri="aa1b21cb-23df-461b-8b8e-4aaeac2f3f50"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EB7FAFA6-FDCF-4091-8393-B79695D0D663}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A1BEDE0-383F-4E7C-82F1-5B51AF37BE3A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
@@ -4476,4 +4489,12 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{46AEFCCE-2E3A-4CC4-B95D-A9558D3302B7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>